<commit_message>
SIM: tpi subte — el campo 12 pasa a 'tiempo de drenaje final' (no era la disipación por tanda)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/materias/SIM/entregables/TPI/subte/04-resultados-corridas.xlsx
+++ b/materias/SIM/entregables/TPI/subte/04-resultados-corridas.xlsx
@@ -1236,7 +1236,7 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Tiempo de disipación</t>
+          <t>Tiempo de drenaje final</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1862,17 +1862,17 @@
       </c>
       <c r="AD7" s="5" t="inlineStr">
         <is>
-          <t>E0 Tiempo de disipación</t>
+          <t>E0 Tiempo de drenaje final</t>
         </is>
       </c>
       <c r="AE7" s="5" t="inlineStr">
         <is>
-          <t>E1 Tiempo de disipación</t>
+          <t>E1 Tiempo de drenaje final</t>
         </is>
       </c>
       <c r="AF7" s="5" t="inlineStr">
         <is>
-          <t>Diferencia Tiempo de disipación</t>
+          <t>Diferencia Tiempo de drenaje final</t>
         </is>
       </c>
       <c r="AG7" s="5" t="inlineStr">

</xml_diff>